<commit_message>
fix(equipment): update 71 assets supplier to 4DEM and clear unverified supplier on 138 FA assets
</commit_message>
<xml_diff>
--- a/ข้อมูลครุภัณฑ์/Template_Items_and_Assets_v3.xlsx
+++ b/ข้อมูลครุภัณฑ์/Template_Items_and_Assets_v3.xlsx
@@ -1747,7 +1747,7 @@
         <v>AED 3 Trainer</v>
       </c>
       <c r="K29" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L29" t="str">
         <v>2025-06-28</v>
@@ -1794,7 +1794,7 @@
         <v>AED 3 Trainer</v>
       </c>
       <c r="K30" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L30" t="str">
         <v>2025-06-28</v>
@@ -2217,7 +2217,7 @@
         <v>Amoul Man Pro (AMM-P)</v>
       </c>
       <c r="K39" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L39" t="str">
         <v>2025-06-28</v>
@@ -2264,7 +2264,7 @@
         <v>Amoul Man Pro (AMM-P)</v>
       </c>
       <c r="K40" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L40" t="str">
         <v>2025-06-28</v>
@@ -2311,7 +2311,7 @@
         <v>รุ่นมาตรฐาน (ปีงบ 68)</v>
       </c>
       <c r="K41" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v>4DEM</v>
       </c>
       <c r="L41" t="str">
         <v>2026-05-01</v>
@@ -2358,7 +2358,7 @@
         <v>รุ่นมาตรฐาน (ปีงบ 68)</v>
       </c>
       <c r="K42" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v>4DEM</v>
       </c>
       <c r="L42" t="str">
         <v>2026-05-01</v>
@@ -2405,7 +2405,7 @@
         <v>รุ่นมาตรฐาน (ปีงบ 68)</v>
       </c>
       <c r="K43" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v>4DEM</v>
       </c>
       <c r="L43" t="str">
         <v>2026-05-01</v>
@@ -2452,7 +2452,7 @@
         <v>รุ่นมาตรฐาน (ปีงบ 68)</v>
       </c>
       <c r="K44" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v>4DEM</v>
       </c>
       <c r="L44" t="str">
         <v>2026-05-01</v>
@@ -2499,7 +2499,7 @@
         <v>รุ่นมาตรฐาน (ปีงบ 68)</v>
       </c>
       <c r="K45" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v>4DEM</v>
       </c>
       <c r="L45" t="str">
         <v>2026-05-01</v>
@@ -2687,7 +2687,7 @@
         <v>Baby CPR Light-indicator</v>
       </c>
       <c r="K49" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L49" t="str">
         <v>2025-06-28</v>
@@ -2734,7 +2734,7 @@
         <v>Baby CPR Light-indicator</v>
       </c>
       <c r="K50" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L50" t="str">
         <v>2025-06-28</v>
@@ -2875,7 +2875,7 @@
         <v>M155</v>
       </c>
       <c r="K53" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L53" t="str">
         <v>2025-06-28</v>
@@ -3580,7 +3580,7 @@
         <v>P93SPC-S</v>
       </c>
       <c r="K68" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L68" t="str">
         <v>2025-06-28</v>
@@ -3627,7 +3627,7 @@
         <v>P93SPC-S</v>
       </c>
       <c r="K69" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L69" t="str">
         <v>2025-06-28</v>
@@ -3674,7 +3674,7 @@
         <v>P93SPC-S</v>
       </c>
       <c r="K70" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L70" t="str">
         <v>2025-06-28</v>
@@ -4191,7 +4191,7 @@
         <v>40201</v>
       </c>
       <c r="K81" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L81" t="str">
         <v>2025-06-28</v>
@@ -5084,7 +5084,7 @@
         <v>LF01043</v>
       </c>
       <c r="K100" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L100" t="str">
         <v>2025-06-28</v>
@@ -5131,7 +5131,7 @@
         <v>LF01043</v>
       </c>
       <c r="K101" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L101" t="str">
         <v>2025-06-28</v>
@@ -6729,7 +6729,7 @@
         <v>CPR Board (CPR-B)</v>
       </c>
       <c r="K135" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L135" t="str">
         <v>2025-06-28</v>
@@ -8985,7 +8985,7 @@
         <v>ไฟฟ้า 3 ไกร์ ราวสไลด์</v>
       </c>
       <c r="K183" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v>4DEM</v>
       </c>
       <c r="L183" t="str">
         <v>2026-05-01</v>
@@ -9032,7 +9032,7 @@
         <v>ไฟฟ้า 3 ไกร์ ราวสไลด์</v>
       </c>
       <c r="K184" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v>4DEM</v>
       </c>
       <c r="L184" t="str">
         <v>2026-05-01</v>
@@ -9079,7 +9079,7 @@
         <v>ไฟฟ้า 3 ไกร์ ราวสไลด์</v>
       </c>
       <c r="K185" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v>4DEM</v>
       </c>
       <c r="L185" t="str">
         <v>2026-05-01</v>
@@ -9126,7 +9126,7 @@
         <v>ไฟฟ้า 3 ไกร์ ราวสไลด์</v>
       </c>
       <c r="K186" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v>4DEM</v>
       </c>
       <c r="L186" t="str">
         <v>2026-05-01</v>
@@ -9173,7 +9173,7 @@
         <v>ไฟฟ้า 3 ไกร์ ราวสไลด์</v>
       </c>
       <c r="K187" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v>4DEM</v>
       </c>
       <c r="L187" t="str">
         <v>2026-05-01</v>
@@ -9220,7 +9220,7 @@
         <v>ไฟฟ้า 3 ไกร์ ราวสไลด์</v>
       </c>
       <c r="K188" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v>4DEM</v>
       </c>
       <c r="L188" t="str">
         <v>2026-05-01</v>
@@ -9267,7 +9267,7 @@
         <v>ไฟฟ้า 3 ไกร์ ราวสไลด์</v>
       </c>
       <c r="K189" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v>4DEM</v>
       </c>
       <c r="L189" t="str">
         <v>2026-05-01</v>
@@ -9314,7 +9314,7 @@
         <v>ไฟฟ้า 3 ไกร์ ราวสไลด์</v>
       </c>
       <c r="K190" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v>4DEM</v>
       </c>
       <c r="L190" t="str">
         <v>2026-05-01</v>
@@ -9361,7 +9361,7 @@
         <v>ไฟฟ้า 3 ไกร์ ราวสไลด์</v>
       </c>
       <c r="K191" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v>4DEM</v>
       </c>
       <c r="L191" t="str">
         <v>2026-05-01</v>
@@ -9408,7 +9408,7 @@
         <v>ไฟฟ้า 3 ไกร์ ราวสไลด์</v>
       </c>
       <c r="K192" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v>4DEM</v>
       </c>
       <c r="L192" t="str">
         <v>2026-05-01</v>
@@ -9455,7 +9455,7 @@
         <v>ไฟฟ้า 3 ไกร์ ราวสไลด์</v>
       </c>
       <c r="K193" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v>4DEM</v>
       </c>
       <c r="L193" t="str">
         <v>2026-05-01</v>
@@ -9502,7 +9502,7 @@
         <v>ไฟฟ้า 3 ไกร์ ราวสไลด์</v>
       </c>
       <c r="K194" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v>4DEM</v>
       </c>
       <c r="L194" t="str">
         <v>2026-05-01</v>
@@ -9549,7 +9549,7 @@
         <v>ไฟฟ้า 3 ไกร์ ราวสไลด์</v>
       </c>
       <c r="K195" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v>4DEM</v>
       </c>
       <c r="L195" t="str">
         <v>2026-05-01</v>
@@ -9596,7 +9596,7 @@
         <v>ไฟฟ้า 3 ไกร์ ราวสไลด์</v>
       </c>
       <c r="K196" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v>4DEM</v>
       </c>
       <c r="L196" t="str">
         <v>2026-05-01</v>
@@ -9643,7 +9643,7 @@
         <v>ไฟฟ้า 3 ไกร์ ราวสไลด์</v>
       </c>
       <c r="K197" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v>4DEM</v>
       </c>
       <c r="L197" t="str">
         <v>2026-05-01</v>
@@ -9690,7 +9690,7 @@
         <v>ไฟฟ้า 3 ไกร์ ราวสไลด์</v>
       </c>
       <c r="K198" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v>4DEM</v>
       </c>
       <c r="L198" t="str">
         <v>2026-05-01</v>
@@ -9737,7 +9737,7 @@
         <v>ไฟฟ้า 3 ไกร์ ราวสไลด์</v>
       </c>
       <c r="K199" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v>4DEM</v>
       </c>
       <c r="L199" t="str">
         <v>2026-05-01</v>
@@ -9784,7 +9784,7 @@
         <v>ไฟฟ้า 3 ไกร์ ราวสไลด์</v>
       </c>
       <c r="K200" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v>4DEM</v>
       </c>
       <c r="L200" t="str">
         <v>2026-05-01</v>
@@ -9831,7 +9831,7 @@
         <v>ไฟฟ้า 3 ไกร์ ราวสไลด์</v>
       </c>
       <c r="K201" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v>4DEM</v>
       </c>
       <c r="L201" t="str">
         <v>2026-05-01</v>
@@ -9878,7 +9878,7 @@
         <v>ไฟฟ้า 3 ไกร์ ราวสไลด์</v>
       </c>
       <c r="K202" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v>4DEM</v>
       </c>
       <c r="L202" t="str">
         <v>2026-05-01</v>
@@ -9925,7 +9925,7 @@
         <v>ไฟฟ้า 2 ไกร์ ราวสไลด์</v>
       </c>
       <c r="K203" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v>4DEM</v>
       </c>
       <c r="L203" t="str">
         <v>2026-05-01</v>
@@ -9972,7 +9972,7 @@
         <v>รุ่นมาตรฐาน</v>
       </c>
       <c r="K204" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v>4DEM</v>
       </c>
       <c r="L204" t="str">
         <v>2026-05-01</v>
@@ -10019,7 +10019,7 @@
         <v>รุ่นมาตรฐาน</v>
       </c>
       <c r="K205" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v>4DEM</v>
       </c>
       <c r="L205" t="str">
         <v>2026-05-01</v>
@@ -10066,7 +10066,7 @@
         <v>P93-Male</v>
       </c>
       <c r="K206" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v>4DEM</v>
       </c>
       <c r="L206" t="str">
         <v>2026-05-01</v>
@@ -10113,7 +10113,7 @@
         <v>P93-Male</v>
       </c>
       <c r="K207" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v>4DEM</v>
       </c>
       <c r="L207" t="str">
         <v>2026-05-01</v>
@@ -10160,7 +10160,7 @@
         <v>P93-Male</v>
       </c>
       <c r="K208" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v>4DEM</v>
       </c>
       <c r="L208" t="str">
         <v>2026-05-01</v>
@@ -10207,7 +10207,7 @@
         <v>P93-Male</v>
       </c>
       <c r="K209" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v>4DEM</v>
       </c>
       <c r="L209" t="str">
         <v>2026-05-01</v>
@@ -10254,7 +10254,7 @@
         <v>P93-Male</v>
       </c>
       <c r="K210" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v>4DEM</v>
       </c>
       <c r="L210" t="str">
         <v>2026-05-01</v>
@@ -10301,7 +10301,7 @@
         <v>P93-Female</v>
       </c>
       <c r="K211" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v>4DEM</v>
       </c>
       <c r="L211" t="str">
         <v>2026-05-01</v>
@@ -10348,7 +10348,7 @@
         <v>P93-Female</v>
       </c>
       <c r="K212" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v>4DEM</v>
       </c>
       <c r="L212" t="str">
         <v>2026-05-01</v>
@@ -10395,7 +10395,7 @@
         <v>P93-Female</v>
       </c>
       <c r="K213" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v>4DEM</v>
       </c>
       <c r="L213" t="str">
         <v>2026-05-01</v>
@@ -10442,7 +10442,7 @@
         <v>P93-Female</v>
       </c>
       <c r="K214" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v>4DEM</v>
       </c>
       <c r="L214" t="str">
         <v>2026-05-01</v>
@@ -10489,7 +10489,7 @@
         <v>P93-Female</v>
       </c>
       <c r="K215" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v>4DEM</v>
       </c>
       <c r="L215" t="str">
         <v>2026-05-01</v>
@@ -10536,7 +10536,7 @@
         <v>รุ่นมาตรฐาน</v>
       </c>
       <c r="K216" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v>4DEM</v>
       </c>
       <c r="L216" t="str">
         <v>2026-05-01</v>
@@ -10583,7 +10583,7 @@
         <v>รุ่นมาตรฐาน</v>
       </c>
       <c r="K217" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v>4DEM</v>
       </c>
       <c r="L217" t="str">
         <v>2026-05-01</v>
@@ -10630,7 +10630,7 @@
         <v>รุ่นมาตรฐาน</v>
       </c>
       <c r="K218" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v>4DEM</v>
       </c>
       <c r="L218" t="str">
         <v>2026-05-01</v>
@@ -10677,7 +10677,7 @@
         <v>รุ่นมาตรฐาน</v>
       </c>
       <c r="K219" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v>4DEM</v>
       </c>
       <c r="L219" t="str">
         <v>2026-05-01</v>
@@ -10724,7 +10724,7 @@
         <v>รุ่นมาตรฐาน</v>
       </c>
       <c r="K220" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v>4DEM</v>
       </c>
       <c r="L220" t="str">
         <v>2026-05-01</v>
@@ -10771,7 +10771,7 @@
         <v>Nursing Manikin Standard</v>
       </c>
       <c r="K221" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v>4DEM</v>
       </c>
       <c r="L221" t="str">
         <v>2026-05-01</v>
@@ -10818,7 +10818,7 @@
         <v>LF00698 Venipuncture Arm</v>
       </c>
       <c r="K222" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L222" t="str">
         <v>2025-06-28</v>
@@ -10865,7 +10865,7 @@
         <v>LF00698 Venipuncture Arm</v>
       </c>
       <c r="K223" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L223" t="str">
         <v>2025-06-28</v>
@@ -10912,7 +10912,7 @@
         <v>LF00698 Venipuncture Arm</v>
       </c>
       <c r="K224" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L224" t="str">
         <v>2025-06-28</v>
@@ -10959,7 +10959,7 @@
         <v>LF00698 Venipuncture Arm</v>
       </c>
       <c r="K225" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L225" t="str">
         <v>2025-06-28</v>
@@ -11006,7 +11006,7 @@
         <v>LF00698 Venipuncture Arm</v>
       </c>
       <c r="K226" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v>4DEM</v>
       </c>
       <c r="L226" t="str">
         <v>2026-05-01</v>
@@ -11053,7 +11053,7 @@
         <v>LF00698 Venipuncture Arm</v>
       </c>
       <c r="K227" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v>4DEM</v>
       </c>
       <c r="L227" t="str">
         <v>2026-05-01</v>
@@ -11100,7 +11100,7 @@
         <v>LF00698 Venipuncture Arm</v>
       </c>
       <c r="K228" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v>4DEM</v>
       </c>
       <c r="L228" t="str">
         <v>2026-05-01</v>
@@ -11147,7 +11147,7 @@
         <v>LF00698 Venipuncture Arm</v>
       </c>
       <c r="K229" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v>4DEM</v>
       </c>
       <c r="L229" t="str">
         <v>2026-05-01</v>
@@ -11194,7 +11194,7 @@
         <v>LF00698 Venipuncture Arm</v>
       </c>
       <c r="K230" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v>4DEM</v>
       </c>
       <c r="L230" t="str">
         <v>2026-05-01</v>
@@ -11241,7 +11241,7 @@
         <v>LF00698 Venipuncture Arm</v>
       </c>
       <c r="K231" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v>4DEM</v>
       </c>
       <c r="L231" t="str">
         <v>2026-05-01</v>
@@ -11288,7 +11288,7 @@
         <v>LF00698 Venipuncture Arm</v>
       </c>
       <c r="K232" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v>4DEM</v>
       </c>
       <c r="L232" t="str">
         <v>2026-05-01</v>
@@ -11335,7 +11335,7 @@
         <v>P100 Wound Care</v>
       </c>
       <c r="K233" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v>4DEM</v>
       </c>
       <c r="L233" t="str">
         <v>2026-05-01</v>
@@ -11382,7 +11382,7 @@
         <v>P100 Wound Care</v>
       </c>
       <c r="K234" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v>4DEM</v>
       </c>
       <c r="L234" t="str">
         <v>2026-05-01</v>
@@ -11429,7 +11429,7 @@
         <v>P100 Wound Care</v>
       </c>
       <c r="K235" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v>4DEM</v>
       </c>
       <c r="L235" t="str">
         <v>2026-05-01</v>
@@ -11476,7 +11476,7 @@
         <v>P100 Wound Care</v>
       </c>
       <c r="K236" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v>4DEM</v>
       </c>
       <c r="L236" t="str">
         <v>2026-05-01</v>
@@ -11523,7 +11523,7 @@
         <v>P100 Wound Care</v>
       </c>
       <c r="K237" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v>4DEM</v>
       </c>
       <c r="L237" t="str">
         <v>2026-05-01</v>
@@ -11570,7 +11570,7 @@
         <v>M155-Wearable</v>
       </c>
       <c r="K238" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v>4DEM</v>
       </c>
       <c r="L238" t="str">
         <v>2026-05-01</v>
@@ -11617,7 +11617,7 @@
         <v>M155-Wearable</v>
       </c>
       <c r="K239" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v>4DEM</v>
       </c>
       <c r="L239" t="str">
         <v>2026-05-01</v>
@@ -11664,7 +11664,7 @@
         <v>M155-Wearable</v>
       </c>
       <c r="K240" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v>4DEM</v>
       </c>
       <c r="L240" t="str">
         <v>2026-05-01</v>
@@ -11711,7 +11711,7 @@
         <v>M155-Wearable</v>
       </c>
       <c r="K241" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v>4DEM</v>
       </c>
       <c r="L241" t="str">
         <v>2026-05-01</v>
@@ -11758,7 +11758,7 @@
         <v>M155-Wearable</v>
       </c>
       <c r="K242" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v>4DEM</v>
       </c>
       <c r="L242" t="str">
         <v>2026-05-01</v>
@@ -11805,7 +11805,7 @@
         <v>Nursing Manikin Standard</v>
       </c>
       <c r="K243" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v>4DEM</v>
       </c>
       <c r="L243" t="str">
         <v>2026-05-01</v>
@@ -11852,7 +11852,7 @@
         <v>Nursing Manikin Standard</v>
       </c>
       <c r="K244" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v>4DEM</v>
       </c>
       <c r="L244" t="str">
         <v>2026-05-01</v>
@@ -11899,7 +11899,7 @@
         <v>Nursing Manikin Standard</v>
       </c>
       <c r="K245" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v>4DEM</v>
       </c>
       <c r="L245" t="str">
         <v>2026-05-01</v>
@@ -11946,7 +11946,7 @@
         <v>Nursing Manikin Standard</v>
       </c>
       <c r="K246" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v>4DEM</v>
       </c>
       <c r="L246" t="str">
         <v>2026-05-01</v>
@@ -11993,7 +11993,7 @@
         <v>Nursing Manikin Standard</v>
       </c>
       <c r="K247" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v>4DEM</v>
       </c>
       <c r="L247" t="str">
         <v>2026-05-01</v>
@@ -12040,7 +12040,7 @@
         <v>Nursing Manikin Standard</v>
       </c>
       <c r="K248" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v>4DEM</v>
       </c>
       <c r="L248" t="str">
         <v>2026-05-01</v>
@@ -12087,7 +12087,7 @@
         <v>Nursing Manikin Standard</v>
       </c>
       <c r="K249" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v>4DEM</v>
       </c>
       <c r="L249" t="str">
         <v>2026-05-01</v>
@@ -12134,7 +12134,7 @@
         <v>Nursing Manikin Standard</v>
       </c>
       <c r="K250" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v>4DEM</v>
       </c>
       <c r="L250" t="str">
         <v>2026-05-01</v>
@@ -12181,7 +12181,7 @@
         <v>Nursing Manikin Standard</v>
       </c>
       <c r="K251" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v>4DEM</v>
       </c>
       <c r="L251" t="str">
         <v>2026-05-01</v>
@@ -12228,7 +12228,7 @@
         <v>Nursing Manikin Standard</v>
       </c>
       <c r="K252" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v>4DEM</v>
       </c>
       <c r="L252" t="str">
         <v>2026-05-01</v>
@@ -12275,7 +12275,7 @@
         <v>Anatomical Model Standard</v>
       </c>
       <c r="K253" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L253" t="str">
         <v>2025-06-28</v>
@@ -12322,7 +12322,7 @@
         <v>Anatomical Model Standard</v>
       </c>
       <c r="K254" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L254" t="str">
         <v>2025-06-28</v>
@@ -12369,7 +12369,7 @@
         <v>Anatomical Model Standard</v>
       </c>
       <c r="K255" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L255" t="str">
         <v>2025-06-28</v>
@@ -12416,7 +12416,7 @@
         <v>Anatomical Model Standard</v>
       </c>
       <c r="K256" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L256" t="str">
         <v>2025-06-28</v>
@@ -12463,7 +12463,7 @@
         <v>Nursing Manikin Standard</v>
       </c>
       <c r="K257" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L257" t="str">
         <v>2025-06-28</v>
@@ -12510,7 +12510,7 @@
         <v>Nursing Manikin Standard</v>
       </c>
       <c r="K258" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L258" t="str">
         <v>2025-06-28</v>
@@ -12557,7 +12557,7 @@
         <v>Nursing Manikin Standard</v>
       </c>
       <c r="K259" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L259" t="str">
         <v>2025-06-28</v>
@@ -12604,7 +12604,7 @@
         <v>Nursing Manikin Standard</v>
       </c>
       <c r="K260" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L260" t="str">
         <v>2025-06-28</v>
@@ -12651,7 +12651,7 @@
         <v>Nursing Manikin Standard</v>
       </c>
       <c r="K261" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L261" t="str">
         <v>2025-06-28</v>
@@ -12698,7 +12698,7 @@
         <v>Nursing Manikin Standard</v>
       </c>
       <c r="K262" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L262" t="str">
         <v>2025-06-28</v>
@@ -12745,7 +12745,7 @@
         <v>หุ่น ครุภัณฑ์และอุปกรณ์ในห้องปฏิบัติการพยาบาลการเรียนรู้แบบเสมือนจริง</v>
       </c>
       <c r="K263" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L263" t="str">
         <v>2025-06-28</v>
@@ -12792,7 +12792,7 @@
         <v>P100 Wound Care</v>
       </c>
       <c r="K264" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L264" t="str">
         <v>2025-06-28</v>
@@ -12839,7 +12839,7 @@
         <v>P100 Wound Care</v>
       </c>
       <c r="K265" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L265" t="str">
         <v>2025-06-28</v>
@@ -12886,7 +12886,7 @@
         <v>Birthing Simulator</v>
       </c>
       <c r="K266" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L266" t="str">
         <v>2025-06-28</v>
@@ -12933,7 +12933,7 @@
         <v>Birthing Simulator</v>
       </c>
       <c r="K267" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L267" t="str">
         <v>2025-06-28</v>
@@ -12980,7 +12980,7 @@
         <v>Birthing Simulator</v>
       </c>
       <c r="K268" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L268" t="str">
         <v>2025-06-28</v>
@@ -13027,7 +13027,7 @@
         <v>Birthing Simulator</v>
       </c>
       <c r="K269" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L269" t="str">
         <v>2025-06-28</v>
@@ -13074,7 +13074,7 @@
         <v>Birthing Simulator</v>
       </c>
       <c r="K270" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L270" t="str">
         <v>2025-06-28</v>
@@ -13121,7 +13121,7 @@
         <v>Obstetric Examination Simulator</v>
       </c>
       <c r="K271" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L271" t="str">
         <v>2025-06-28</v>
@@ -13168,7 +13168,7 @@
         <v>Obstetric Examination Simulator</v>
       </c>
       <c r="K272" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L272" t="str">
         <v>2025-06-28</v>
@@ -13215,7 +13215,7 @@
         <v>Baby Care Simulator</v>
       </c>
       <c r="K273" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L273" t="str">
         <v>2025-06-28</v>
@@ -13262,7 +13262,7 @@
         <v>Baby Care Simulator</v>
       </c>
       <c r="K274" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L274" t="str">
         <v>2025-06-28</v>
@@ -13309,7 +13309,7 @@
         <v>Baby Care Simulator</v>
       </c>
       <c r="K275" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L275" t="str">
         <v>2025-06-28</v>
@@ -13356,7 +13356,7 @@
         <v>Baby Care Simulator</v>
       </c>
       <c r="K276" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L276" t="str">
         <v>2025-06-28</v>
@@ -13403,7 +13403,7 @@
         <v>Baby Care Simulator</v>
       </c>
       <c r="K277" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L277" t="str">
         <v>2025-06-28</v>
@@ -13450,7 +13450,7 @@
         <v>718-8804 SAM</v>
       </c>
       <c r="K278" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L278" t="str">
         <v>2025-06-28</v>
@@ -13497,7 +13497,7 @@
         <v>Home Visit Bag Set</v>
       </c>
       <c r="K279" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L279" t="str">
         <v>2025-06-28</v>
@@ -13544,7 +13544,7 @@
         <v>Home Visit Bag Set</v>
       </c>
       <c r="K280" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L280" t="str">
         <v>2025-06-28</v>
@@ -13591,7 +13591,7 @@
         <v>Home Visit Bag Set</v>
       </c>
       <c r="K281" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L281" t="str">
         <v>2025-06-28</v>
@@ -13638,7 +13638,7 @@
         <v>Hospital Bed Standard</v>
       </c>
       <c r="K282" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L282" t="str">
         <v>2025-06-28</v>
@@ -13685,7 +13685,7 @@
         <v>มือหมุน 3 ไกร์</v>
       </c>
       <c r="K283" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L283" t="str">
         <v>2025-06-28</v>
@@ -13732,7 +13732,7 @@
         <v>มือหมุน 3 ไกร์</v>
       </c>
       <c r="K284" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L284" t="str">
         <v>2025-06-28</v>
@@ -13779,7 +13779,7 @@
         <v>มือหมุน 3 ไกร์</v>
       </c>
       <c r="K285" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L285" t="str">
         <v>2025-06-28</v>
@@ -13826,7 +13826,7 @@
         <v>มือหมุน 3 ไกร์</v>
       </c>
       <c r="K286" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L286" t="str">
         <v>2025-06-28</v>
@@ -13873,7 +13873,7 @@
         <v>มือหมุน 3 ไกร์</v>
       </c>
       <c r="K287" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L287" t="str">
         <v>2025-06-28</v>
@@ -13920,7 +13920,7 @@
         <v>มือหมุน 3 ไกร์</v>
       </c>
       <c r="K288" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L288" t="str">
         <v>2025-06-28</v>
@@ -13967,7 +13967,7 @@
         <v>มือหมุน 3 ไกร์</v>
       </c>
       <c r="K289" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L289" t="str">
         <v>2025-06-28</v>
@@ -14014,7 +14014,7 @@
         <v>มือหมุน 3 ไกร์</v>
       </c>
       <c r="K290" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L290" t="str">
         <v>2025-06-28</v>
@@ -14061,7 +14061,7 @@
         <v>มือหมุน 3 ไกร์</v>
       </c>
       <c r="K291" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L291" t="str">
         <v>2025-06-28</v>
@@ -14108,7 +14108,7 @@
         <v>เตียงทำคลอด 2 ตอนปรับระดับ</v>
       </c>
       <c r="K292" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L292" t="str">
         <v>2025-06-28</v>
@@ -14155,7 +14155,7 @@
         <v>เตียงเด็กอ่อนพร้อมเบาะ</v>
       </c>
       <c r="K293" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L293" t="str">
         <v>2025-06-28</v>
@@ -14202,7 +14202,7 @@
         <v>เตียงเด็กอ่อนพร้อมเบาะ</v>
       </c>
       <c r="K294" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L294" t="str">
         <v>2025-06-28</v>
@@ -14249,7 +14249,7 @@
         <v>Bedside Cabinet</v>
       </c>
       <c r="K295" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L295" t="str">
         <v>2025-06-28</v>
@@ -14296,7 +14296,7 @@
         <v>Bedside Cabinet</v>
       </c>
       <c r="K296" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L296" t="str">
         <v>2025-06-28</v>
@@ -14343,7 +14343,7 @@
         <v>Bedside Cabinet</v>
       </c>
       <c r="K297" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L297" t="str">
         <v>2025-06-28</v>
@@ -14390,7 +14390,7 @@
         <v>Bedside Cabinet</v>
       </c>
       <c r="K298" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L298" t="str">
         <v>2025-06-28</v>
@@ -14437,7 +14437,7 @@
         <v>Bedside Cabinet</v>
       </c>
       <c r="K299" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L299" t="str">
         <v>2025-06-28</v>
@@ -14484,7 +14484,7 @@
         <v>Bedside Cabinet</v>
       </c>
       <c r="K300" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L300" t="str">
         <v>2025-06-28</v>
@@ -14531,7 +14531,7 @@
         <v>Bedside Cabinet</v>
       </c>
       <c r="K301" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L301" t="str">
         <v>2025-06-28</v>
@@ -14578,7 +14578,7 @@
         <v>Bedside Cabinet</v>
       </c>
       <c r="K302" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L302" t="str">
         <v>2025-06-28</v>
@@ -14625,7 +14625,7 @@
         <v>Overbed Table</v>
       </c>
       <c r="K303" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L303" t="str">
         <v>2025-06-28</v>
@@ -14672,7 +14672,7 @@
         <v>Overbed Table</v>
       </c>
       <c r="K304" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L304" t="str">
         <v>2025-06-28</v>
@@ -14719,7 +14719,7 @@
         <v>Overbed Table</v>
       </c>
       <c r="K305" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L305" t="str">
         <v>2025-06-28</v>
@@ -14766,7 +14766,7 @@
         <v>Overbed Table</v>
       </c>
       <c r="K306" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L306" t="str">
         <v>2025-06-28</v>
@@ -14813,7 +14813,7 @@
         <v>Overbed Table</v>
       </c>
       <c r="K307" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L307" t="str">
         <v>2025-06-28</v>
@@ -14860,7 +14860,7 @@
         <v>Overbed Table</v>
       </c>
       <c r="K308" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L308" t="str">
         <v>2025-06-28</v>
@@ -14907,7 +14907,7 @@
         <v>Overbed Table</v>
       </c>
       <c r="K309" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L309" t="str">
         <v>2025-06-28</v>
@@ -14954,7 +14954,7 @@
         <v>Overbed Table</v>
       </c>
       <c r="K310" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L310" t="str">
         <v>2025-06-28</v>
@@ -15001,7 +15001,7 @@
         <v>Medical Cart Standard</v>
       </c>
       <c r="K311" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L311" t="str">
         <v>2025-06-28</v>
@@ -15048,7 +15048,7 @@
         <v>Medical Cart Standard</v>
       </c>
       <c r="K312" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L312" t="str">
         <v>2025-06-28</v>
@@ -15095,7 +15095,7 @@
         <v>Medical Cart Standard</v>
       </c>
       <c r="K313" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L313" t="str">
         <v>2025-06-28</v>
@@ -15142,7 +15142,7 @@
         <v>Medical Cart Standard</v>
       </c>
       <c r="K314" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L314" t="str">
         <v>2025-06-28</v>
@@ -15189,7 +15189,7 @@
         <v>Medical Cart Standard</v>
       </c>
       <c r="K315" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L315" t="str">
         <v>2025-06-28</v>
@@ -15236,7 +15236,7 @@
         <v>Medical Cart Standard</v>
       </c>
       <c r="K316" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L316" t="str">
         <v>2025-06-28</v>
@@ -15283,7 +15283,7 @@
         <v>Medical Cart Standard</v>
       </c>
       <c r="K317" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L317" t="str">
         <v>2025-06-28</v>
@@ -15330,7 +15330,7 @@
         <v>Medical Cart Standard</v>
       </c>
       <c r="K318" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L318" t="str">
         <v>2025-06-28</v>
@@ -15377,7 +15377,7 @@
         <v>Medical Device Standard</v>
       </c>
       <c r="K319" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L319" t="str">
         <v>2025-06-28</v>
@@ -15424,7 +15424,7 @@
         <v>Stainless Waste Bin</v>
       </c>
       <c r="K320" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L320" t="str">
         <v>2025-06-28</v>
@@ -15471,7 +15471,7 @@
         <v>Stainless Waste Bin</v>
       </c>
       <c r="K321" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L321" t="str">
         <v>2025-06-28</v>
@@ -15518,7 +15518,7 @@
         <v>Stainless Waste Bin</v>
       </c>
       <c r="K322" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L322" t="str">
         <v>2025-06-28</v>
@@ -15565,7 +15565,7 @@
         <v>Stainless Waste Bin</v>
       </c>
       <c r="K323" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L323" t="str">
         <v>2025-06-28</v>
@@ -15612,7 +15612,7 @@
         <v>Stainless Waste Bin</v>
       </c>
       <c r="K324" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L324" t="str">
         <v>2025-06-28</v>
@@ -15659,7 +15659,7 @@
         <v>Stainless Waste Bin</v>
       </c>
       <c r="K325" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L325" t="str">
         <v>2025-06-28</v>
@@ -15706,7 +15706,7 @@
         <v>Stainless Waste Bin</v>
       </c>
       <c r="K326" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L326" t="str">
         <v>2025-06-28</v>
@@ -15753,7 +15753,7 @@
         <v>Stainless Waste Bin</v>
       </c>
       <c r="K327" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L327" t="str">
         <v>2025-06-28</v>
@@ -15800,7 +15800,7 @@
         <v>Medical Device Standard</v>
       </c>
       <c r="K328" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L328" t="str">
         <v>2025-06-28</v>
@@ -15847,7 +15847,7 @@
         <v>Medical Device Standard</v>
       </c>
       <c r="K329" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L329" t="str">
         <v>2025-06-28</v>
@@ -15894,7 +15894,7 @@
         <v>Mercurial Sphygmomanometer</v>
       </c>
       <c r="K330" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L330" t="str">
         <v>2025-06-28</v>
@@ -15941,7 +15941,7 @@
         <v>Mercurial Sphygmomanometer</v>
       </c>
       <c r="K331" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L331" t="str">
         <v>2025-06-28</v>
@@ -15988,7 +15988,7 @@
         <v>Mercurial Sphygmomanometer</v>
       </c>
       <c r="K332" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L332" t="str">
         <v>2025-06-28</v>
@@ -16035,7 +16035,7 @@
         <v>Mercurial Sphygmomanometer</v>
       </c>
       <c r="K333" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L333" t="str">
         <v>2025-06-28</v>
@@ -16082,7 +16082,7 @@
         <v>Mercurial Sphygmomanometer</v>
       </c>
       <c r="K334" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L334" t="str">
         <v>2025-06-28</v>
@@ -16129,7 +16129,7 @@
         <v>Digital BP Monitor</v>
       </c>
       <c r="K335" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L335" t="str">
         <v>2025-06-28</v>
@@ -16176,7 +16176,7 @@
         <v>Digital BP Monitor</v>
       </c>
       <c r="K336" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L336" t="str">
         <v>2025-06-28</v>
@@ -16223,7 +16223,7 @@
         <v>Digital BP Monitor</v>
       </c>
       <c r="K337" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L337" t="str">
         <v>2025-06-28</v>
@@ -16270,7 +16270,7 @@
         <v>Digital BP Monitor</v>
       </c>
       <c r="K338" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L338" t="str">
         <v>2025-06-28</v>
@@ -16317,7 +16317,7 @@
         <v>Digital BP Monitor</v>
       </c>
       <c r="K339" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L339" t="str">
         <v>2025-06-28</v>
@@ -16364,7 +16364,7 @@
         <v>Digital BP Monitor</v>
       </c>
       <c r="K340" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L340" t="str">
         <v>2025-06-28</v>
@@ -16411,7 +16411,7 @@
         <v>Digital BP Monitor</v>
       </c>
       <c r="K341" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L341" t="str">
         <v>2025-06-28</v>
@@ -16458,7 +16458,7 @@
         <v>Digital BP Monitor</v>
       </c>
       <c r="K342" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L342" t="str">
         <v>2025-06-28</v>
@@ -16505,7 +16505,7 @@
         <v>Digital BP Monitor</v>
       </c>
       <c r="K343" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L343" t="str">
         <v>2025-06-28</v>
@@ -16552,7 +16552,7 @@
         <v>Digital BP Monitor</v>
       </c>
       <c r="K344" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L344" t="str">
         <v>2025-06-28</v>
@@ -16599,7 +16599,7 @@
         <v>Medical Device Standard</v>
       </c>
       <c r="K345" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L345" t="str">
         <v>2025-06-28</v>
@@ -16646,7 +16646,7 @@
         <v>Medical Device Standard</v>
       </c>
       <c r="K346" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L346" t="str">
         <v>2025-06-28</v>
@@ -16693,7 +16693,7 @@
         <v>Medical Device Standard</v>
       </c>
       <c r="K347" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L347" t="str">
         <v>2025-06-28</v>
@@ -16740,7 +16740,7 @@
         <v>DT-Otoscope</v>
       </c>
       <c r="K348" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L348" t="str">
         <v>2025-06-28</v>
@@ -16787,7 +16787,7 @@
         <v>DT-Ophthalmoscope</v>
       </c>
       <c r="K349" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L349" t="str">
         <v>2025-06-28</v>
@@ -16834,7 +16834,7 @@
         <v>Laryngoscope Set</v>
       </c>
       <c r="K350" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L350" t="str">
         <v>2025-06-28</v>
@@ -16881,7 +16881,7 @@
         <v>Patient Transfer Slide</v>
       </c>
       <c r="K351" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L351" t="str">
         <v>2025-06-28</v>
@@ -16928,7 +16928,7 @@
         <v>Patient Transfer Slide</v>
       </c>
       <c r="K352" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L352" t="str">
         <v>2025-06-28</v>
@@ -16975,7 +16975,7 @@
         <v>Medical Device Standard</v>
       </c>
       <c r="K353" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L353" t="str">
         <v>2025-06-28</v>
@@ -17022,7 +17022,7 @@
         <v>Medical Device Standard</v>
       </c>
       <c r="K354" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L354" t="str">
         <v>2025-06-28</v>
@@ -17069,7 +17069,7 @@
         <v>Medical Device Standard</v>
       </c>
       <c r="K355" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L355" t="str">
         <v>2025-06-28</v>
@@ -17116,7 +17116,7 @@
         <v>Medical Device Standard</v>
       </c>
       <c r="K356" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L356" t="str">
         <v>2025-06-28</v>
@@ -17163,7 +17163,7 @@
         <v>Medical Device Standard</v>
       </c>
       <c r="K357" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L357" t="str">
         <v>2025-06-28</v>
@@ -17210,7 +17210,7 @@
         <v>Medical Device Standard</v>
       </c>
       <c r="K358" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L358" t="str">
         <v>2025-06-28</v>
@@ -17257,7 +17257,7 @@
         <v>Medical Device Standard</v>
       </c>
       <c r="K359" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L359" t="str">
         <v>2025-06-28</v>
@@ -17304,7 +17304,7 @@
         <v>Medical Device Standard</v>
       </c>
       <c r="K360" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L360" t="str">
         <v>2025-06-28</v>
@@ -17351,7 +17351,7 @@
         <v>Medical Device Standard</v>
       </c>
       <c r="K361" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L361" t="str">
         <v>2025-06-28</v>
@@ -17398,7 +17398,7 @@
         <v>Medical Device Standard</v>
       </c>
       <c r="K362" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L362" t="str">
         <v>2025-06-28</v>
@@ -17445,7 +17445,7 @@
         <v>Massage Chair</v>
       </c>
       <c r="K363" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L363" t="str">
         <v>2025-06-28</v>
@@ -17492,7 +17492,7 @@
         <v>Massage Chair</v>
       </c>
       <c r="K364" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L364" t="str">
         <v>2025-06-28</v>
@@ -17633,7 +17633,7 @@
         <v>IV Stand Stainless</v>
       </c>
       <c r="K367" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L367" t="str">
         <v>2025-06-28</v>
@@ -17680,7 +17680,7 @@
         <v>IV Stand Stainless</v>
       </c>
       <c r="K368" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L368" t="str">
         <v>2025-06-28</v>
@@ -17727,7 +17727,7 @@
         <v>IV Stand Stainless</v>
       </c>
       <c r="K369" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L369" t="str">
         <v>2025-06-28</v>
@@ -17774,7 +17774,7 @@
         <v>IV Stand Stainless</v>
       </c>
       <c r="K370" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L370" t="str">
         <v>2025-06-28</v>
@@ -17821,7 +17821,7 @@
         <v>IV Stand Stainless</v>
       </c>
       <c r="K371" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L371" t="str">
         <v>2025-06-28</v>
@@ -17868,7 +17868,7 @@
         <v>IV Stand Stainless</v>
       </c>
       <c r="K372" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L372" t="str">
         <v>2025-06-28</v>
@@ -17915,7 +17915,7 @@
         <v>IV Stand Stainless</v>
       </c>
       <c r="K373" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L373" t="str">
         <v>2025-06-28</v>
@@ -17962,7 +17962,7 @@
         <v>IV Stand Stainless</v>
       </c>
       <c r="K374" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
+        <v/>
       </c>
       <c r="L374" t="str">
         <v>2025-06-28</v>

</xml_diff>

<commit_message>
fix(equipment): update brand and model for 14 specific items per user verification
</commit_message>
<xml_diff>
--- a/ข้อมูลครุภัณฑ์/Template_Items_and_Assets_v3.xlsx
+++ b/ข้อมูลครุภัณฑ์/Template_Items_and_Assets_v3.xlsx
@@ -2305,10 +2305,10 @@
         <v>2025-05-01</v>
       </c>
       <c r="I41" t="str">
-        <v>Amoul</v>
+        <v>Prestan พรีสแตน</v>
       </c>
       <c r="J41" t="str">
-        <v>รุ่นมาตรฐาน (ปีงบ 68)</v>
+        <v>PP AM 100M MS</v>
       </c>
       <c r="K41" t="str">
         <v>4DEM</v>
@@ -2352,10 +2352,10 @@
         <v>2025-05-01</v>
       </c>
       <c r="I42" t="str">
-        <v>Amoul</v>
+        <v>Prestan พรีสแตน</v>
       </c>
       <c r="J42" t="str">
-        <v>รุ่นมาตรฐาน (ปีงบ 68)</v>
+        <v>PP AM 100M MS</v>
       </c>
       <c r="K42" t="str">
         <v>4DEM</v>
@@ -2399,10 +2399,10 @@
         <v>2025-05-01</v>
       </c>
       <c r="I43" t="str">
-        <v>Amoul</v>
+        <v>Prestan พรีสแตน</v>
       </c>
       <c r="J43" t="str">
-        <v>รุ่นมาตรฐาน (ปีงบ 68)</v>
+        <v>PP AM 100M MS</v>
       </c>
       <c r="K43" t="str">
         <v>4DEM</v>
@@ -2446,10 +2446,10 @@
         <v>2025-05-01</v>
       </c>
       <c r="I44" t="str">
-        <v>Amoul</v>
+        <v>Prestan พรีสแตน</v>
       </c>
       <c r="J44" t="str">
-        <v>รุ่นมาตรฐาน (ปีงบ 68)</v>
+        <v>PP AM 100M MS</v>
       </c>
       <c r="K44" t="str">
         <v>4DEM</v>
@@ -2493,10 +2493,10 @@
         <v>2025-05-01</v>
       </c>
       <c r="I45" t="str">
-        <v>Amoul</v>
+        <v>Prestan พรีสแตน</v>
       </c>
       <c r="J45" t="str">
-        <v>รุ่นมาตรฐาน (ปีงบ 68)</v>
+        <v>PP AM 100M MS</v>
       </c>
       <c r="K45" t="str">
         <v>4DEM</v>
@@ -5172,10 +5172,10 @@
         <v>2025-08-19</v>
       </c>
       <c r="I102" t="str">
-        <v>Nasco Life/form</v>
+        <v>อัพไรท์ ซิมมูเลชั่น</v>
       </c>
       <c r="J102" t="str">
-        <v>LF01043</v>
+        <v>800-816</v>
       </c>
       <c r="K102" t="str">
         <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
@@ -5219,10 +5219,10 @@
         <v>2025-08-19</v>
       </c>
       <c r="I103" t="str">
-        <v>Nasco Life/form</v>
+        <v>อัพไรท์ ซิมมูเลชั่น</v>
       </c>
       <c r="J103" t="str">
-        <v>LF01043</v>
+        <v>800-816</v>
       </c>
       <c r="K103" t="str">
         <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
@@ -5266,10 +5266,10 @@
         <v>2025-08-19</v>
       </c>
       <c r="I104" t="str">
-        <v>Nasco Life/form</v>
+        <v>อัพไรท์ ซิมมูเลชั่น</v>
       </c>
       <c r="J104" t="str">
-        <v>LF01043</v>
+        <v>800-816</v>
       </c>
       <c r="K104" t="str">
         <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
@@ -5313,10 +5313,10 @@
         <v>2025-08-19</v>
       </c>
       <c r="I105" t="str">
-        <v>Nasco Life/form</v>
+        <v>อัพไรท์ ซิมมูเลชั่น</v>
       </c>
       <c r="J105" t="str">
-        <v>LF01043</v>
+        <v>800-816</v>
       </c>
       <c r="K105" t="str">
         <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
@@ -5360,10 +5360,10 @@
         <v>2025-08-19</v>
       </c>
       <c r="I106" t="str">
-        <v>Nasco Life/form</v>
+        <v>อัพไรท์ ซิมมูเลชั่น</v>
       </c>
       <c r="J106" t="str">
-        <v>LF01043</v>
+        <v>800-816</v>
       </c>
       <c r="K106" t="str">
         <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
@@ -5407,10 +5407,10 @@
         <v>2025-08-19</v>
       </c>
       <c r="I107" t="str">
-        <v>Nasco Life/form</v>
+        <v>อัพไรท์ ซิมมูเลชั่น</v>
       </c>
       <c r="J107" t="str">
-        <v>LF01043</v>
+        <v>800-816</v>
       </c>
       <c r="K107" t="str">
         <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
@@ -5454,10 +5454,10 @@
         <v>2025-08-19</v>
       </c>
       <c r="I108" t="str">
-        <v>Nasco Life/form</v>
+        <v>อัพไรท์ ซิมมูเลชั่น</v>
       </c>
       <c r="J108" t="str">
-        <v>LF01043</v>
+        <v>800-816</v>
       </c>
       <c r="K108" t="str">
         <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
@@ -5501,10 +5501,10 @@
         <v>2025-08-19</v>
       </c>
       <c r="I109" t="str">
-        <v>Nasco Life/form</v>
+        <v>อัพไรท์ ซิมมูเลชั่น</v>
       </c>
       <c r="J109" t="str">
-        <v>LF01043</v>
+        <v>800-816</v>
       </c>
       <c r="K109" t="str">
         <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
@@ -5548,10 +5548,10 @@
         <v>2025-08-19</v>
       </c>
       <c r="I110" t="str">
-        <v>Nasco Life/form</v>
+        <v>อัพไรท์ ซิมมูเลชั่น</v>
       </c>
       <c r="J110" t="str">
-        <v>LF01043</v>
+        <v>800-816</v>
       </c>
       <c r="K110" t="str">
         <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
@@ -5595,10 +5595,10 @@
         <v>2025-08-19</v>
       </c>
       <c r="I111" t="str">
-        <v>Nasco Life/form</v>
+        <v>อัพไรท์ ซิมมูเลชั่น</v>
       </c>
       <c r="J111" t="str">
-        <v>LF01043</v>
+        <v>800-816</v>
       </c>
       <c r="K111" t="str">
         <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
@@ -9919,10 +9919,10 @@
         <v>2025-05-01</v>
       </c>
       <c r="I203" t="str">
-        <v>Upright Simulation</v>
+        <v>เตียงเฟาร์เลอร์ 2 ไกร์</v>
       </c>
       <c r="J203" t="str">
-        <v>ไฟฟ้า 2 ไกร์ ราวสไลด์</v>
+        <v>แบบ ดิจิตอล</v>
       </c>
       <c r="K203" t="str">
         <v>4DEM</v>
@@ -9966,10 +9966,10 @@
         <v>2025-05-01</v>
       </c>
       <c r="I204" t="str">
-        <v>Upright Simulation</v>
+        <v>4DEM</v>
       </c>
       <c r="J204" t="str">
-        <v>รุ่นมาตรฐาน</v>
+        <v>หุ่น SIM MAN Gaumard Scientific</v>
       </c>
       <c r="K204" t="str">
         <v>4DEM</v>
@@ -10013,10 +10013,10 @@
         <v>2025-05-01</v>
       </c>
       <c r="I205" t="str">
-        <v>Upright Simulation</v>
+        <v>4DEM</v>
       </c>
       <c r="J205" t="str">
-        <v>รุ่นมาตรฐาน</v>
+        <v>Qube AVPro</v>
       </c>
       <c r="K205" t="str">
         <v>4DEM</v>
@@ -10060,10 +10060,10 @@
         <v>2025-05-01</v>
       </c>
       <c r="I206" t="str">
-        <v>3B Scientific</v>
+        <v>Limbs &amp; Things</v>
       </c>
       <c r="J206" t="str">
-        <v>P93-Male</v>
+        <v>60850</v>
       </c>
       <c r="K206" t="str">
         <v>4DEM</v>
@@ -10107,10 +10107,10 @@
         <v>2025-05-01</v>
       </c>
       <c r="I207" t="str">
-        <v>3B Scientific</v>
+        <v>Limbs &amp; Things</v>
       </c>
       <c r="J207" t="str">
-        <v>P93-Male</v>
+        <v>60850</v>
       </c>
       <c r="K207" t="str">
         <v>4DEM</v>
@@ -10154,10 +10154,10 @@
         <v>2025-05-01</v>
       </c>
       <c r="I208" t="str">
-        <v>3B Scientific</v>
+        <v>Limbs &amp; Things</v>
       </c>
       <c r="J208" t="str">
-        <v>P93-Male</v>
+        <v>60850</v>
       </c>
       <c r="K208" t="str">
         <v>4DEM</v>
@@ -10201,10 +10201,10 @@
         <v>2025-05-01</v>
       </c>
       <c r="I209" t="str">
-        <v>3B Scientific</v>
+        <v>Limbs &amp; Things</v>
       </c>
       <c r="J209" t="str">
-        <v>P93-Male</v>
+        <v>60850</v>
       </c>
       <c r="K209" t="str">
         <v>4DEM</v>
@@ -10248,10 +10248,10 @@
         <v>2025-05-01</v>
       </c>
       <c r="I210" t="str">
-        <v>3B Scientific</v>
+        <v>Limbs &amp; Things</v>
       </c>
       <c r="J210" t="str">
-        <v>P93-Male</v>
+        <v>60850</v>
       </c>
       <c r="K210" t="str">
         <v>4DEM</v>
@@ -10295,10 +10295,10 @@
         <v>2025-05-01</v>
       </c>
       <c r="I211" t="str">
-        <v>3B Scientific</v>
+        <v>Limbs &amp; Things</v>
       </c>
       <c r="J211" t="str">
-        <v>P93-Female</v>
+        <v>60851</v>
       </c>
       <c r="K211" t="str">
         <v>4DEM</v>
@@ -10342,10 +10342,10 @@
         <v>2025-05-01</v>
       </c>
       <c r="I212" t="str">
-        <v>3B Scientific</v>
+        <v>Limbs &amp; Things</v>
       </c>
       <c r="J212" t="str">
-        <v>P93-Female</v>
+        <v>60851</v>
       </c>
       <c r="K212" t="str">
         <v>4DEM</v>
@@ -10389,10 +10389,10 @@
         <v>2025-05-01</v>
       </c>
       <c r="I213" t="str">
-        <v>3B Scientific</v>
+        <v>Limbs &amp; Things</v>
       </c>
       <c r="J213" t="str">
-        <v>P93-Female</v>
+        <v>60851</v>
       </c>
       <c r="K213" t="str">
         <v>4DEM</v>
@@ -10436,10 +10436,10 @@
         <v>2025-05-01</v>
       </c>
       <c r="I214" t="str">
-        <v>3B Scientific</v>
+        <v>Limbs &amp; Things</v>
       </c>
       <c r="J214" t="str">
-        <v>P93-Female</v>
+        <v>60851</v>
       </c>
       <c r="K214" t="str">
         <v>4DEM</v>
@@ -10483,10 +10483,10 @@
         <v>2025-05-01</v>
       </c>
       <c r="I215" t="str">
-        <v>3B Scientific</v>
+        <v>Limbs &amp; Things</v>
       </c>
       <c r="J215" t="str">
-        <v>P93-Female</v>
+        <v>60851</v>
       </c>
       <c r="K215" t="str">
         <v>4DEM</v>
@@ -10530,10 +10530,10 @@
         <v>2025-05-01</v>
       </c>
       <c r="I216" t="str">
-        <v>Upright Simulation</v>
+        <v>KOKEN</v>
       </c>
       <c r="J216" t="str">
-        <v>รุ่นมาตรฐาน</v>
+        <v>LM-097B</v>
       </c>
       <c r="K216" t="str">
         <v>4DEM</v>
@@ -10577,10 +10577,10 @@
         <v>2025-05-01</v>
       </c>
       <c r="I217" t="str">
-        <v>Upright Simulation</v>
+        <v>KOKEN</v>
       </c>
       <c r="J217" t="str">
-        <v>รุ่นมาตรฐาน</v>
+        <v>LM-097B</v>
       </c>
       <c r="K217" t="str">
         <v>4DEM</v>
@@ -10624,10 +10624,10 @@
         <v>2025-05-01</v>
       </c>
       <c r="I218" t="str">
-        <v>Upright Simulation</v>
+        <v>KOKEN</v>
       </c>
       <c r="J218" t="str">
-        <v>รุ่นมาตรฐาน</v>
+        <v>LM-097B</v>
       </c>
       <c r="K218" t="str">
         <v>4DEM</v>
@@ -10671,10 +10671,10 @@
         <v>2025-05-01</v>
       </c>
       <c r="I219" t="str">
-        <v>Upright Simulation</v>
+        <v>KOKEN</v>
       </c>
       <c r="J219" t="str">
-        <v>รุ่นมาตรฐาน</v>
+        <v>LM-097B</v>
       </c>
       <c r="K219" t="str">
         <v>4DEM</v>
@@ -10718,10 +10718,10 @@
         <v>2025-05-01</v>
       </c>
       <c r="I220" t="str">
-        <v>Upright Simulation</v>
+        <v>KOKEN</v>
       </c>
       <c r="J220" t="str">
-        <v>รุ่นมาตรฐาน</v>
+        <v>LM-097B</v>
       </c>
       <c r="K220" t="str">
         <v>4DEM</v>
@@ -10741,7 +10741,7 @@
     </row>
     <row r="221">
       <c r="A221" t="str">
-        <v>หุ่นจำลองผู้ใหญ่</v>
+        <v>หุ่นจำลองผู้ใหญ่ (SIM MAN)</v>
       </c>
       <c r="B221" t="str">
         <v>EQ-FMS-0003</v>
@@ -10765,10 +10765,10 @@
         <v>2025-05-01</v>
       </c>
       <c r="I221" t="str">
-        <v>3B Scientific</v>
+        <v>Gaumard Scientific</v>
       </c>
       <c r="J221" t="str">
-        <v>Nursing Manikin Standard</v>
+        <v>S3201.PK</v>
       </c>
       <c r="K221" t="str">
         <v>4DEM</v>
@@ -11000,10 +11000,10 @@
         <v>2025-05-01</v>
       </c>
       <c r="I226" t="str">
-        <v>Nasco Life/form</v>
+        <v>Koken</v>
       </c>
       <c r="J226" t="str">
-        <v>LF00698 Venipuncture Arm</v>
+        <v>LM-028</v>
       </c>
       <c r="K226" t="str">
         <v>4DEM</v>
@@ -11047,10 +11047,10 @@
         <v>2025-05-01</v>
       </c>
       <c r="I227" t="str">
-        <v>Nasco Life/form</v>
+        <v>Koken</v>
       </c>
       <c r="J227" t="str">
-        <v>LF00698 Venipuncture Arm</v>
+        <v>LM-028</v>
       </c>
       <c r="K227" t="str">
         <v>4DEM</v>
@@ -11094,10 +11094,10 @@
         <v>2025-05-01</v>
       </c>
       <c r="I228" t="str">
-        <v>Nasco Life/form</v>
+        <v>Koken</v>
       </c>
       <c r="J228" t="str">
-        <v>LF00698 Venipuncture Arm</v>
+        <v>LM-028</v>
       </c>
       <c r="K228" t="str">
         <v>4DEM</v>
@@ -11141,10 +11141,10 @@
         <v>2025-05-01</v>
       </c>
       <c r="I229" t="str">
-        <v>Nasco Life/form</v>
+        <v>Koken</v>
       </c>
       <c r="J229" t="str">
-        <v>LF00698 Venipuncture Arm</v>
+        <v>LM-028</v>
       </c>
       <c r="K229" t="str">
         <v>4DEM</v>
@@ -11188,10 +11188,10 @@
         <v>2025-05-01</v>
       </c>
       <c r="I230" t="str">
-        <v>Nasco Life/form</v>
+        <v>Koken</v>
       </c>
       <c r="J230" t="str">
-        <v>LF00698 Venipuncture Arm</v>
+        <v>LM-028</v>
       </c>
       <c r="K230" t="str">
         <v>4DEM</v>
@@ -11235,10 +11235,10 @@
         <v>2025-05-01</v>
       </c>
       <c r="I231" t="str">
-        <v>Nasco Life/form</v>
+        <v>Koken</v>
       </c>
       <c r="J231" t="str">
-        <v>LF00698 Venipuncture Arm</v>
+        <v>LM-028</v>
       </c>
       <c r="K231" t="str">
         <v>4DEM</v>
@@ -11282,10 +11282,10 @@
         <v>2025-05-01</v>
       </c>
       <c r="I232" t="str">
-        <v>Nasco Life/form</v>
+        <v>Koken</v>
       </c>
       <c r="J232" t="str">
-        <v>LF00698 Venipuncture Arm</v>
+        <v>LM-028</v>
       </c>
       <c r="K232" t="str">
         <v>4DEM</v>
@@ -11329,10 +11329,10 @@
         <v>2025-05-01</v>
       </c>
       <c r="I233" t="str">
-        <v>3B Scientific</v>
+        <v>Nasco Healthcare</v>
       </c>
       <c r="J233" t="str">
-        <v>P100 Wound Care</v>
+        <v>LF00929U</v>
       </c>
       <c r="K233" t="str">
         <v>4DEM</v>
@@ -11376,10 +11376,10 @@
         <v>2025-05-01</v>
       </c>
       <c r="I234" t="str">
-        <v>3B Scientific</v>
+        <v>Nasco Healthcare</v>
       </c>
       <c r="J234" t="str">
-        <v>P100 Wound Care</v>
+        <v>LF00929U</v>
       </c>
       <c r="K234" t="str">
         <v>4DEM</v>
@@ -11423,10 +11423,10 @@
         <v>2025-05-01</v>
       </c>
       <c r="I235" t="str">
-        <v>3B Scientific</v>
+        <v>Nasco Healthcare</v>
       </c>
       <c r="J235" t="str">
-        <v>P100 Wound Care</v>
+        <v>LF00929U</v>
       </c>
       <c r="K235" t="str">
         <v>4DEM</v>
@@ -11470,10 +11470,10 @@
         <v>2025-05-01</v>
       </c>
       <c r="I236" t="str">
-        <v>3B Scientific</v>
+        <v>Nasco Healthcare</v>
       </c>
       <c r="J236" t="str">
-        <v>P100 Wound Care</v>
+        <v>LF00929U</v>
       </c>
       <c r="K236" t="str">
         <v>4DEM</v>
@@ -11517,10 +11517,10 @@
         <v>2025-05-01</v>
       </c>
       <c r="I237" t="str">
-        <v>3B Scientific</v>
+        <v>Nasco Healthcare</v>
       </c>
       <c r="J237" t="str">
-        <v>P100 Wound Care</v>
+        <v>LF00929U</v>
       </c>
       <c r="K237" t="str">
         <v>4DEM</v>
@@ -11564,10 +11564,10 @@
         <v>2025-05-01</v>
       </c>
       <c r="I238" t="str">
-        <v>Koken</v>
+        <v>4DEM</v>
       </c>
       <c r="J238" t="str">
-        <v>M155-Wearable</v>
+        <v>L-IMD</v>
       </c>
       <c r="K238" t="str">
         <v>4DEM</v>
@@ -11611,10 +11611,10 @@
         <v>2025-05-01</v>
       </c>
       <c r="I239" t="str">
-        <v>Koken</v>
+        <v>4DEM</v>
       </c>
       <c r="J239" t="str">
-        <v>M155-Wearable</v>
+        <v>L-IMD</v>
       </c>
       <c r="K239" t="str">
         <v>4DEM</v>
@@ -11658,10 +11658,10 @@
         <v>2025-05-01</v>
       </c>
       <c r="I240" t="str">
-        <v>Koken</v>
+        <v>4DEM</v>
       </c>
       <c r="J240" t="str">
-        <v>M155-Wearable</v>
+        <v>L-IMD</v>
       </c>
       <c r="K240" t="str">
         <v>4DEM</v>
@@ -11705,10 +11705,10 @@
         <v>2025-05-01</v>
       </c>
       <c r="I241" t="str">
-        <v>Koken</v>
+        <v>4DEM</v>
       </c>
       <c r="J241" t="str">
-        <v>M155-Wearable</v>
+        <v>L-IMD</v>
       </c>
       <c r="K241" t="str">
         <v>4DEM</v>
@@ -11752,10 +11752,10 @@
         <v>2025-05-01</v>
       </c>
       <c r="I242" t="str">
-        <v>Koken</v>
+        <v>4DEM</v>
       </c>
       <c r="J242" t="str">
-        <v>M155-Wearable</v>
+        <v>L-IMD</v>
       </c>
       <c r="K242" t="str">
         <v>4DEM</v>
@@ -11799,10 +11799,10 @@
         <v>2025-05-01</v>
       </c>
       <c r="I243" t="str">
-        <v>3B Scientific</v>
+        <v>CLA Nursing Doll</v>
       </c>
       <c r="J243" t="str">
-        <v>Nursing Manikin Standard</v>
+        <v>CLA 1M</v>
       </c>
       <c r="K243" t="str">
         <v>4DEM</v>
@@ -11846,10 +11846,10 @@
         <v>2025-05-01</v>
       </c>
       <c r="I244" t="str">
-        <v>3B Scientific</v>
+        <v>CLA Nursing Doll</v>
       </c>
       <c r="J244" t="str">
-        <v>Nursing Manikin Standard</v>
+        <v>CLA 1M</v>
       </c>
       <c r="K244" t="str">
         <v>4DEM</v>
@@ -11893,10 +11893,10 @@
         <v>2025-05-01</v>
       </c>
       <c r="I245" t="str">
-        <v>3B Scientific</v>
+        <v>CLA Nursing Doll</v>
       </c>
       <c r="J245" t="str">
-        <v>Nursing Manikin Standard</v>
+        <v>CLA 1M</v>
       </c>
       <c r="K245" t="str">
         <v>4DEM</v>
@@ -11940,10 +11940,10 @@
         <v>2025-05-01</v>
       </c>
       <c r="I246" t="str">
-        <v>3B Scientific</v>
+        <v>CLA Nursing Doll</v>
       </c>
       <c r="J246" t="str">
-        <v>Nursing Manikin Standard</v>
+        <v>CLA 1M</v>
       </c>
       <c r="K246" t="str">
         <v>4DEM</v>
@@ -11987,10 +11987,10 @@
         <v>2025-05-01</v>
       </c>
       <c r="I247" t="str">
-        <v>3B Scientific</v>
+        <v>CLA Nursing Doll</v>
       </c>
       <c r="J247" t="str">
-        <v>Nursing Manikin Standard</v>
+        <v>CLA 1M</v>
       </c>
       <c r="K247" t="str">
         <v>4DEM</v>
@@ -12034,10 +12034,10 @@
         <v>2025-05-01</v>
       </c>
       <c r="I248" t="str">
-        <v>3B Scientific</v>
+        <v>CLA Nursing Doll</v>
       </c>
       <c r="J248" t="str">
-        <v>Nursing Manikin Standard</v>
+        <v>CLA 1F</v>
       </c>
       <c r="K248" t="str">
         <v>4DEM</v>
@@ -12081,10 +12081,10 @@
         <v>2025-05-01</v>
       </c>
       <c r="I249" t="str">
-        <v>3B Scientific</v>
+        <v>CLA Nursing Doll</v>
       </c>
       <c r="J249" t="str">
-        <v>Nursing Manikin Standard</v>
+        <v>CLA 1F</v>
       </c>
       <c r="K249" t="str">
         <v>4DEM</v>
@@ -12128,10 +12128,10 @@
         <v>2025-05-01</v>
       </c>
       <c r="I250" t="str">
-        <v>3B Scientific</v>
+        <v>CLA Nursing Doll</v>
       </c>
       <c r="J250" t="str">
-        <v>Nursing Manikin Standard</v>
+        <v>CLA 1F</v>
       </c>
       <c r="K250" t="str">
         <v>4DEM</v>
@@ -12175,10 +12175,10 @@
         <v>2025-05-01</v>
       </c>
       <c r="I251" t="str">
-        <v>3B Scientific</v>
+        <v>CLA Nursing Doll</v>
       </c>
       <c r="J251" t="str">
-        <v>Nursing Manikin Standard</v>
+        <v>CLA 1F</v>
       </c>
       <c r="K251" t="str">
         <v>4DEM</v>
@@ -12222,10 +12222,10 @@
         <v>2025-05-01</v>
       </c>
       <c r="I252" t="str">
-        <v>3B Scientific</v>
+        <v>CLA Nursing Doll</v>
       </c>
       <c r="J252" t="str">
-        <v>Nursing Manikin Standard</v>
+        <v>CLA 1F</v>
       </c>
       <c r="K252" t="str">
         <v>4DEM</v>

</xml_diff>